<commit_message>
fix: compare benchmark workbook account names literally
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F8C752-E7C6-4F43-B097-B819F3C16655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D7584C-0873-4866-91B3-52F7472F520C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27897,11 +27897,11 @@
         <v>PASS</v>
       </c>
       <c r="C5" s="8">
-        <f>SUMPRODUCT((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;""))</f>
+        <f t="array" ref="C5">SUMPRODUCT((MMULT(--(tblPnl[Key]=TRANSPOSE(tblPnl[Key])),ROW(tblPnl[Key])^0)&gt;1)*(tblPnl[Key]&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
+        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((MMULT(--(tblPnl[Key]=TRANSPOSE(tblPnl[Key])),ROW(tblPnl[Key])^0)&gt;1)*(tblPnl[Key]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
         <v/>
       </c>
     </row>
@@ -27914,11 +27914,11 @@
         <v>PASS</v>
       </c>
       <c r="C6" s="8">
-        <f>SUMPRODUCT((COUNTIF(tblMapping[Key],tblMapping[Key])&gt;1)*(tblMapping[Key]&lt;&gt;""))</f>
+        <f t="array" ref="C6">SUMPRODUCT((MMULT(--(tblMapping[Key]=TRANSPOSE(tblMapping[Key])),ROW(tblMapping[Key])^0)&gt;1)*(tblMapping[Key]&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="D6" s="8" t="str">
-        <f t="array" ref="D6">IF(C6=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((COUNTIF(tblMapping[Key],tblMapping[Key])&gt;1)*(tblMapping[Key]&lt;&gt;"")*(ROW(tblMapping[Account])-1)))))</f>
+        <f t="array" ref="D6">IF(C6=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((MMULT(--(tblMapping[Key]=TRANSPOSE(tblMapping[Key])),ROW(tblMapping[Key])^0)&gt;1)*(tblMapping[Key]&lt;&gt;"")*(ROW(tblMapping[Account])-1)))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: compare benchmark workbook account names literally (#174)
Account names containing wildcard characters could be flagged as duplicates even when distinct. The workbook now compares normalised names literally and retains duplicate detection for matching names (F024).

Verification: 321 tests passed, 3 skipped, 93% coverage; Ruff, mypy, dependency audit and build passed. Six native Excel controls pass for *, ? and ~. Only four review formulas changed; other cells and styles match the baseline. Native rendering was inspected.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F8C752-E7C6-4F43-B097-B819F3C16655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D7584C-0873-4866-91B3-52F7472F520C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27897,11 +27897,11 @@
         <v>PASS</v>
       </c>
       <c r="C5" s="8">
-        <f>SUMPRODUCT((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;""))</f>
+        <f t="array" ref="C5">SUMPRODUCT((MMULT(--(tblPnl[Key]=TRANSPOSE(tblPnl[Key])),ROW(tblPnl[Key])^0)&gt;1)*(tblPnl[Key]&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((COUNTIF(tblPnl[Key],tblPnl[Key])&gt;1)*(tblPnl[Key]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
+        <f t="array" ref="D5">IF(C5=0,"",INDEX(tblPnl[Account],SUMPRODUCT(MAX((MMULT(--(tblPnl[Key]=TRANSPOSE(tblPnl[Key])),ROW(tblPnl[Key])^0)&gt;1)*(tblPnl[Key]&lt;&gt;"")*(ROW(tblPnl[Account])-1)))))</f>
         <v/>
       </c>
     </row>
@@ -27914,11 +27914,11 @@
         <v>PASS</v>
       </c>
       <c r="C6" s="8">
-        <f>SUMPRODUCT((COUNTIF(tblMapping[Key],tblMapping[Key])&gt;1)*(tblMapping[Key]&lt;&gt;""))</f>
+        <f t="array" ref="C6">SUMPRODUCT((MMULT(--(tblMapping[Key]=TRANSPOSE(tblMapping[Key])),ROW(tblMapping[Key])^0)&gt;1)*(tblMapping[Key]&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="D6" s="8" t="str">
-        <f t="array" ref="D6">IF(C6=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((COUNTIF(tblMapping[Key],tblMapping[Key])&gt;1)*(tblMapping[Key]&lt;&gt;"")*(ROW(tblMapping[Account])-1)))))</f>
+        <f t="array" ref="D6">IF(C6=0,"",INDEX(tblMapping[Account],SUMPRODUCT(MAX((MMULT(--(tblMapping[Key]=TRANSPOSE(tblMapping[Key])),ROW(tblMapping[Key])^0)&gt;1)*(tblMapping[Key]&lt;&gt;"")*(ROW(tblMapping[Account])-1)))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare five package versions and release notes (#234)
Prepare five package versions and release notes derived from their git history. Align manifests, runtime copies, lockfiles, documentation and workbook version labels.

Add root verification routing and CI coverage. Keep checkout version reporting independent of unrelated installed metadata, with regression tests for stale and absent metadata.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.1.8. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.1.9. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1222,7 +1222,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.8</t>
+    <t>0.1.9</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Fail closed on unknown ratio headings and hold the page file to every industry
The builder stops when a line above a full set of ranges is not a known heading, accepts headings with a missing or accent-typed quote, and refuses to search past the next year heading for bands; four pages that an earlier parse had cut short now contribute 17 more ranges (708 in all). The loader checks business_type_count and that the included and excluded business types account for every industry. The attribution wording says a single printed figure is stored as equal bounds. The workbook was recalculated in desktop Excel.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990E8EE1-090B-4DF9-B3DA-1748D721CD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903EECC8-0800-4006-B205-13B4FD7BFAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5730" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5730" uniqueCount="539">
   <si>
     <t>ATO small business benchmark comparison</t>
   </si>
@@ -1150,9 +1150,6 @@
     <t>84329267f96e25c6e8caaf91704353d914a00f17aa9b68e9b524e6cebb924b2a</t>
   </si>
   <si>
-    <t>labour_to_turnover rent_to_turnover</t>
-  </si>
-  <si>
     <t>be498a47beb7ba82a3ae356e2b11e22725cbc6738f9f15ebfe0fc576956b35b6</t>
   </si>
   <si>
@@ -1174,334 +1171,334 @@
     <t>7293db71d3eafc752c6d460e0d64d7dcf6bdf4bf61bda4a19ebe4cad603727f2</t>
   </si>
   <si>
+    <t>d1964f80c66379dded8c27808c9c6f1f4d50c4a57e0980807b25dbfd45702313</t>
+  </si>
+  <si>
+    <t>2ada353f6212f3c627fb4343a8dfce7f47fad98cc7427214fc4144493b6f2d75</t>
+  </si>
+  <si>
+    <t>c6145ad6f00712a5ee009b81be9281bd7671279c488a68d644dbbddf63674ea9</t>
+  </si>
+  <si>
+    <t>882b8ca16caf8a0454c2c7ccd59e93c9a910c4ddfd56cff24da51ccab60a88e0</t>
+  </si>
+  <si>
+    <t>c12be06e63fcfc61a8375a30a8dc5bba6b748f87ae04d022def0d02431d455d5</t>
+  </si>
+  <si>
+    <t>759d839915a7435366404914ec92731bb097046c1e35cc510fe2c0f82945ee4b</t>
+  </si>
+  <si>
+    <t>f54cb844f220cc786587b2d36c1de1d77bb64a26d73033abb9e637d93ba24e62</t>
+  </si>
+  <si>
+    <t>aeea370676377d67631a50ba9e81cdf90b31cd8cc9d098f0b0f7eb83204110c5</t>
+  </si>
+  <si>
+    <t>eadb798fb991e064387bf1bad68632b8b5d2caaaf2554bca4fe84804a6093211</t>
+  </si>
+  <si>
+    <t>e0ef475d24620a6d632150351c0266739f93ddac7774113c49d3e25183590f32</t>
+  </si>
+  <si>
+    <t>7925078ce24864ffbff8cbaa118627bb113f2d40eba941664f38353bbe34f241</t>
+  </si>
+  <si>
+    <t>e2e1244a773d8922f6fb843164d6e0c5909cfc561aa35e599a3276f8d0141ae8</t>
+  </si>
+  <si>
+    <t>ab901a93d18e50c843643efa8758d4cf310fcc7153a215eb1232ec60683f177e</t>
+  </si>
+  <si>
+    <t>06af80f4ff2538f809adbad1dca378c33478404f7a79a12356d281be36b540c0</t>
+  </si>
+  <si>
+    <t>15779fecf9fac873aa8f86d321a5850fdcb17c3da5c021ee1f33eca14e2f1865</t>
+  </si>
+  <si>
+    <t>adcdba8d9a097c92d04a1be6f34833667dd736cf6a2f724e1d48956ebe712d5e</t>
+  </si>
+  <si>
+    <t>6ed3c26a47460aaa5210bf8882e405f19a948cecd7b85adcb4c15305c0cb7d64</t>
+  </si>
+  <si>
+    <t>1ae312174d151ec3c777c3659e2348fe87761dd3960a354bc0200fac4a64daa3</t>
+  </si>
+  <si>
+    <t>d24fe633805f919ac8a72723db75ba0d0cf11757a2c0b79fe70028488678bc6f</t>
+  </si>
+  <si>
+    <t>4c4c9e49c3ddc5817a8768d2161114be8dea99364fcec0bff850fe093b3a8d3b</t>
+  </si>
+  <si>
+    <t>a6e1b2f1e738963fd195ebf4eeaa6aada095a50672b4f30e764e6e09129791c3</t>
+  </si>
+  <si>
+    <t>7858b6be86e1d8d5d087eb46687124ae3c942ac5fd116788fa8bfc910863707d</t>
+  </si>
+  <si>
+    <t>8da78efaac80db59b511893eadb79b4319de752f964de39ae3169b45f9a55983</t>
+  </si>
+  <si>
+    <t>9d9575421934e13bf00551b7957b56c2eafafa508eec576585d9fefceaac3aa7</t>
+  </si>
+  <si>
+    <t>b19cb3378a33fbe9435ea5e7c2592f8fce031574d53ce43028ab08fbd37fefb3</t>
+  </si>
+  <si>
+    <t>dcbda4d2c6e0baafbf326551403f9e2384f4a2db8dd23ffc64e2cd11810488ab</t>
+  </si>
+  <si>
+    <t>7a3ff1c3c2a6e4c41b31066cecc89bd2e14a2beeb2c0d6325811e5e247b7642c</t>
+  </si>
+  <si>
+    <t>e5e70efdc72cf52f728982b41c617de1aa3ac22c0f233210d7b032beb8c55a3f</t>
+  </si>
+  <si>
+    <t>ee4516c71c899f4319d42056bd7ebdce93c50e8754a94c89aef7c7fbef8a5906</t>
+  </si>
+  <si>
+    <t>52fddc3db577c810ee9b325e1371f0aac9d2ad34d6657dcb40ad5d8813c74b63</t>
+  </si>
+  <si>
+    <t>b2aeecf9d1d3af30eff0bcafd2a658d42f84f847337d9ab63a687079e01247ba</t>
+  </si>
+  <si>
+    <t>ff6910517c64b93034876d2ee64950e6c53431ac1b400c8a3560267b5a92b5dd</t>
+  </si>
+  <si>
+    <t>9e5f4a3405e70097c8ec7dd992283229eede0498d7e4aa6a28d5f9c25d7dde62</t>
+  </si>
+  <si>
+    <t>150abc83cdfa189fefcf94bea9d9d2ae7d25f05254a9b27b3a9b2cc0dbc1b925</t>
+  </si>
+  <si>
+    <t>243ccf23553f31abb5a85e8645309f36ced00478ab516482bdaaa559ef76c4fb</t>
+  </si>
+  <si>
+    <t>8bf7e2db411fcf848e185c71f864ac65af70a549a43f850a9a578cae3a764262</t>
+  </si>
+  <si>
+    <t>74e55f6373a33f9eb60a4a6d3974d80ee202c140c6400186ce5d1649f5484ed1</t>
+  </si>
+  <si>
+    <t>43d5b970b7503c9ca96786fe9583dcdbc436a13c92e2d4354d1264b927d5d788</t>
+  </si>
+  <si>
+    <t>d177040473aa3c80b4e128f220856c50cc9de99d9a42a67fe6c7dd03b3ccc345</t>
+  </si>
+  <si>
+    <t>5305bbc94a9fd4e34d0fe38db0100b2b630df94aa1b8c3a3a078174651ba6030</t>
+  </si>
+  <si>
+    <t>9665f899b877de72332244f7933839e02796abbb6821b3d8e1ad6d010d4aef73</t>
+  </si>
+  <si>
+    <t>55ed6ce6a02c55e4790638c8a423ef2c7564d3dbc0719d911ff1b345081dcdd6</t>
+  </si>
+  <si>
+    <t>39b72db9c16f98b20def69446cf2db5e11b37af9a7f011be176579c747d7ffcd</t>
+  </si>
+  <si>
+    <t>0da114f12aabce001cf0c4f055b45fcedd0a3d5d14f7a1dfd116c690aee3e2bf</t>
+  </si>
+  <si>
+    <t>2c199549b6f8b36fba2821d16b0d1ddc3774fa922bbd4981c8f5d659dfcc7ad6</t>
+  </si>
+  <si>
+    <t>ab97fdc84c879c16d1ae799abf7a5ce91e6f0507c94a650a543a79ec02ad743d</t>
+  </si>
+  <si>
+    <t>025f9042e4b48976f20538dd3dbe8c85c11f1a490ab81243d7e12904218ad90d</t>
+  </si>
+  <si>
+    <t>5ac308bc362d3e0decd6c4a020de174f251dfd42995bbee1894046a2f1f389f8</t>
+  </si>
+  <si>
+    <t>277161e21229e3abf7f8f0b25746957e5450a25b9f2ffc2d3f87ceb798c701a0</t>
+  </si>
+  <si>
+    <t>6b3ab160c29327b68595bd9358cce522a621e8ef3673ad098d7f4629b2de2a7e</t>
+  </si>
+  <si>
+    <t>28f18a013d2006458911dbb8eec249a86bdab456455c074d07a9307564529baa</t>
+  </si>
+  <si>
+    <t>01b92ebf219f4fa033628b5e306ed5e9f445c6a869ae507aeaa7032a2a00cb92</t>
+  </si>
+  <si>
+    <t>cost_of_sales_to_turnover motor_vehicle_to_turnover</t>
+  </si>
+  <si>
+    <t>c261256c79f66895b71eb9f9176b6a63c01c639e70059e806c3dca73c18c498a</t>
+  </si>
+  <si>
+    <t>61f8fafdd74da5d1bf86a07d4e7e8deea5d278a5abb7ec2d74976e5f192db782</t>
+  </si>
+  <si>
+    <t>b177f3d645356cd33522f35774e9e38b5330c8d6f79130b394495d39ba5273bd</t>
+  </si>
+  <si>
+    <t>fe2746729b7af0d683cc68f55d71193fa65d968e62bd22937705ea5db3e58131</t>
+  </si>
+  <si>
+    <t>0220ab956eab909a25ace045a294dfd9372714612d42b48889a6c3550c341a14</t>
+  </si>
+  <si>
+    <t>eae154cd25cb8eb4f091e3a7836d664c61800595ac93ba81d49133630fb8ac38</t>
+  </si>
+  <si>
+    <t>03f5d057e835768a3e1582a8509eb4c16bcf3a002339dcdeeb27d2a6ef806fbc</t>
+  </si>
+  <si>
+    <t>90ec95e1d48c6813bd7842f5040ba737d39ced0e7dc195064393668121156c78</t>
+  </si>
+  <si>
+    <t>b70e502e9b330b343d2c13f0ac2d7c38eff778d12328bd7e38a2db045b588840</t>
+  </si>
+  <si>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>Benchmark year</t>
+  </si>
+  <si>
+    <t>Expenses shown as negatives? (Y/N)</t>
+  </si>
+  <si>
+    <t>Activity statement W1 (blank if not supplied)</t>
+  </si>
+  <si>
+    <t>Expense sign factor</t>
+  </si>
+  <si>
+    <t>Bucket totals (SUMIFS over tblPnl)</t>
+  </si>
+  <si>
+    <t>What the ATO does with it</t>
+  </si>
+  <si>
+    <t>Sales of goods and services. The ATO's turnover label.</t>
+  </si>
+  <si>
+    <t>Business income that is not sales, for example interest or grants.</t>
+  </si>
+  <si>
+    <t>Cost of sales, excluding any salary and wages inside it.</t>
+  </si>
+  <si>
+    <t>Salary and wages included in cost of sales.</t>
+  </si>
+  <si>
+    <t>Salary and wages outside cost of sales.</t>
+  </si>
+  <si>
+    <t>Contractor, subcontractor and commission expenses.</t>
+  </si>
+  <si>
+    <t>Payments to associated persons.</t>
+  </si>
+  <si>
+    <t>Rent expenses.</t>
+  </si>
+  <si>
+    <t>Motor vehicle expenses.</t>
+  </si>
+  <si>
+    <t>Every other expense, including superannuation and depreciation.</t>
+  </si>
+  <si>
+    <t>Not part of the ATO calculation, for example income tax expense.</t>
+  </si>
+  <si>
+    <t>Figures</t>
+  </si>
+  <si>
+    <t>Sales of goods and services</t>
+  </si>
+  <si>
+    <t>Other business income</t>
+  </si>
+  <si>
+    <t>Total business income</t>
+  </si>
+  <si>
+    <t>Turnover</t>
+  </si>
+  <si>
+    <t>Turnover basis</t>
+  </si>
+  <si>
+    <t>Total expenses reported</t>
+  </si>
+  <si>
+    <t>Payments to associated persons</t>
+  </si>
+  <si>
+    <t>Total expenses for ratio</t>
+  </si>
+  <si>
+    <t>Cost of sales for ratio (excludes wages)</t>
+  </si>
+  <si>
+    <t>Salary and wages label (wages + cost of sales wages + associates)</t>
+  </si>
+  <si>
+    <t>Labour base (W1 when it exceeds the label)</t>
+  </si>
+  <si>
+    <t>Labour (base less associates plus contractors and commission)</t>
+  </si>
+  <si>
+    <t>Band lookup (1E9 = no match)</t>
+  </si>
+  <si>
+    <t>Band row in tblBands (0 = none)</t>
+  </si>
+  <si>
+    <t>Turnover band</t>
+  </si>
+  <si>
+    <t>Industry row in tblBands (0 = not published for the year)</t>
+  </si>
+  <si>
+    <t>Published key ratio</t>
+  </si>
+  <si>
+    <t>Key ratio used</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Benchmark min</t>
+  </si>
+  <si>
+    <t>Benchmark max</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Range source</t>
+  </si>
+  <si>
+    <t>Cost of sales to turnover</t>
+  </si>
+  <si>
+    <t>Total expenses to turnover</t>
+  </si>
+  <si>
+    <t>labour_to_turnover</t>
+  </si>
+  <si>
+    <t>Labour to turnover</t>
+  </si>
+  <si>
     <t>rent_to_turnover</t>
-  </si>
-  <si>
-    <t>d1964f80c66379dded8c27808c9c6f1f4d50c4a57e0980807b25dbfd45702313</t>
-  </si>
-  <si>
-    <t>2ada353f6212f3c627fb4343a8dfce7f47fad98cc7427214fc4144493b6f2d75</t>
-  </si>
-  <si>
-    <t>c6145ad6f00712a5ee009b81be9281bd7671279c488a68d644dbbddf63674ea9</t>
-  </si>
-  <si>
-    <t>882b8ca16caf8a0454c2c7ccd59e93c9a910c4ddfd56cff24da51ccab60a88e0</t>
-  </si>
-  <si>
-    <t>c12be06e63fcfc61a8375a30a8dc5bba6b748f87ae04d022def0d02431d455d5</t>
-  </si>
-  <si>
-    <t>759d839915a7435366404914ec92731bb097046c1e35cc510fe2c0f82945ee4b</t>
-  </si>
-  <si>
-    <t>f54cb844f220cc786587b2d36c1de1d77bb64a26d73033abb9e637d93ba24e62</t>
-  </si>
-  <si>
-    <t>aeea370676377d67631a50ba9e81cdf90b31cd8cc9d098f0b0f7eb83204110c5</t>
-  </si>
-  <si>
-    <t>eadb798fb991e064387bf1bad68632b8b5d2caaaf2554bca4fe84804a6093211</t>
-  </si>
-  <si>
-    <t>e0ef475d24620a6d632150351c0266739f93ddac7774113c49d3e25183590f32</t>
-  </si>
-  <si>
-    <t>7925078ce24864ffbff8cbaa118627bb113f2d40eba941664f38353bbe34f241</t>
-  </si>
-  <si>
-    <t>e2e1244a773d8922f6fb843164d6e0c5909cfc561aa35e599a3276f8d0141ae8</t>
-  </si>
-  <si>
-    <t>ab901a93d18e50c843643efa8758d4cf310fcc7153a215eb1232ec60683f177e</t>
-  </si>
-  <si>
-    <t>06af80f4ff2538f809adbad1dca378c33478404f7a79a12356d281be36b540c0</t>
-  </si>
-  <si>
-    <t>15779fecf9fac873aa8f86d321a5850fdcb17c3da5c021ee1f33eca14e2f1865</t>
-  </si>
-  <si>
-    <t>adcdba8d9a097c92d04a1be6f34833667dd736cf6a2f724e1d48956ebe712d5e</t>
-  </si>
-  <si>
-    <t>6ed3c26a47460aaa5210bf8882e405f19a948cecd7b85adcb4c15305c0cb7d64</t>
-  </si>
-  <si>
-    <t>1ae312174d151ec3c777c3659e2348fe87761dd3960a354bc0200fac4a64daa3</t>
-  </si>
-  <si>
-    <t>d24fe633805f919ac8a72723db75ba0d0cf11757a2c0b79fe70028488678bc6f</t>
-  </si>
-  <si>
-    <t>4c4c9e49c3ddc5817a8768d2161114be8dea99364fcec0bff850fe093b3a8d3b</t>
-  </si>
-  <si>
-    <t>a6e1b2f1e738963fd195ebf4eeaa6aada095a50672b4f30e764e6e09129791c3</t>
-  </si>
-  <si>
-    <t>7858b6be86e1d8d5d087eb46687124ae3c942ac5fd116788fa8bfc910863707d</t>
-  </si>
-  <si>
-    <t>8da78efaac80db59b511893eadb79b4319de752f964de39ae3169b45f9a55983</t>
-  </si>
-  <si>
-    <t>9d9575421934e13bf00551b7957b56c2eafafa508eec576585d9fefceaac3aa7</t>
-  </si>
-  <si>
-    <t>b19cb3378a33fbe9435ea5e7c2592f8fce031574d53ce43028ab08fbd37fefb3</t>
-  </si>
-  <si>
-    <t>dcbda4d2c6e0baafbf326551403f9e2384f4a2db8dd23ffc64e2cd11810488ab</t>
-  </si>
-  <si>
-    <t>7a3ff1c3c2a6e4c41b31066cecc89bd2e14a2beeb2c0d6325811e5e247b7642c</t>
-  </si>
-  <si>
-    <t>e5e70efdc72cf52f728982b41c617de1aa3ac22c0f233210d7b032beb8c55a3f</t>
-  </si>
-  <si>
-    <t>ee4516c71c899f4319d42056bd7ebdce93c50e8754a94c89aef7c7fbef8a5906</t>
-  </si>
-  <si>
-    <t>52fddc3db577c810ee9b325e1371f0aac9d2ad34d6657dcb40ad5d8813c74b63</t>
-  </si>
-  <si>
-    <t>b2aeecf9d1d3af30eff0bcafd2a658d42f84f847337d9ab63a687079e01247ba</t>
-  </si>
-  <si>
-    <t>ff6910517c64b93034876d2ee64950e6c53431ac1b400c8a3560267b5a92b5dd</t>
-  </si>
-  <si>
-    <t>9e5f4a3405e70097c8ec7dd992283229eede0498d7e4aa6a28d5f9c25d7dde62</t>
-  </si>
-  <si>
-    <t>150abc83cdfa189fefcf94bea9d9d2ae7d25f05254a9b27b3a9b2cc0dbc1b925</t>
-  </si>
-  <si>
-    <t>243ccf23553f31abb5a85e8645309f36ced00478ab516482bdaaa559ef76c4fb</t>
-  </si>
-  <si>
-    <t>8bf7e2db411fcf848e185c71f864ac65af70a549a43f850a9a578cae3a764262</t>
-  </si>
-  <si>
-    <t>74e55f6373a33f9eb60a4a6d3974d80ee202c140c6400186ce5d1649f5484ed1</t>
-  </si>
-  <si>
-    <t>43d5b970b7503c9ca96786fe9583dcdbc436a13c92e2d4354d1264b927d5d788</t>
-  </si>
-  <si>
-    <t>d177040473aa3c80b4e128f220856c50cc9de99d9a42a67fe6c7dd03b3ccc345</t>
-  </si>
-  <si>
-    <t>5305bbc94a9fd4e34d0fe38db0100b2b630df94aa1b8c3a3a078174651ba6030</t>
-  </si>
-  <si>
-    <t>9665f899b877de72332244f7933839e02796abbb6821b3d8e1ad6d010d4aef73</t>
-  </si>
-  <si>
-    <t>55ed6ce6a02c55e4790638c8a423ef2c7564d3dbc0719d911ff1b345081dcdd6</t>
-  </si>
-  <si>
-    <t>39b72db9c16f98b20def69446cf2db5e11b37af9a7f011be176579c747d7ffcd</t>
-  </si>
-  <si>
-    <t>0da114f12aabce001cf0c4f055b45fcedd0a3d5d14f7a1dfd116c690aee3e2bf</t>
-  </si>
-  <si>
-    <t>2c199549b6f8b36fba2821d16b0d1ddc3774fa922bbd4981c8f5d659dfcc7ad6</t>
-  </si>
-  <si>
-    <t>ab97fdc84c879c16d1ae799abf7a5ce91e6f0507c94a650a543a79ec02ad743d</t>
-  </si>
-  <si>
-    <t>025f9042e4b48976f20538dd3dbe8c85c11f1a490ab81243d7e12904218ad90d</t>
-  </si>
-  <si>
-    <t>5ac308bc362d3e0decd6c4a020de174f251dfd42995bbee1894046a2f1f389f8</t>
-  </si>
-  <si>
-    <t>277161e21229e3abf7f8f0b25746957e5450a25b9f2ffc2d3f87ceb798c701a0</t>
-  </si>
-  <si>
-    <t>6b3ab160c29327b68595bd9358cce522a621e8ef3673ad098d7f4629b2de2a7e</t>
-  </si>
-  <si>
-    <t>28f18a013d2006458911dbb8eec249a86bdab456455c074d07a9307564529baa</t>
-  </si>
-  <si>
-    <t>01b92ebf219f4fa033628b5e306ed5e9f445c6a869ae507aeaa7032a2a00cb92</t>
-  </si>
-  <si>
-    <t>cost_of_sales_to_turnover motor_vehicle_to_turnover</t>
-  </si>
-  <si>
-    <t>c261256c79f66895b71eb9f9176b6a63c01c639e70059e806c3dca73c18c498a</t>
-  </si>
-  <si>
-    <t>61f8fafdd74da5d1bf86a07d4e7e8deea5d278a5abb7ec2d74976e5f192db782</t>
-  </si>
-  <si>
-    <t>b177f3d645356cd33522f35774e9e38b5330c8d6f79130b394495d39ba5273bd</t>
-  </si>
-  <si>
-    <t>fe2746729b7af0d683cc68f55d71193fa65d968e62bd22937705ea5db3e58131</t>
-  </si>
-  <si>
-    <t>0220ab956eab909a25ace045a294dfd9372714612d42b48889a6c3550c341a14</t>
-  </si>
-  <si>
-    <t>eae154cd25cb8eb4f091e3a7836d664c61800595ac93ba81d49133630fb8ac38</t>
-  </si>
-  <si>
-    <t>03f5d057e835768a3e1582a8509eb4c16bcf3a002339dcdeeb27d2a6ef806fbc</t>
-  </si>
-  <si>
-    <t>90ec95e1d48c6813bd7842f5040ba737d39ced0e7dc195064393668121156c78</t>
-  </si>
-  <si>
-    <t>b70e502e9b330b343d2c13f0ac2d7c38eff778d12328bd7e38a2db045b588840</t>
-  </si>
-  <si>
-    <t>Inputs</t>
-  </si>
-  <si>
-    <t>Benchmark year</t>
-  </si>
-  <si>
-    <t>Expenses shown as negatives? (Y/N)</t>
-  </si>
-  <si>
-    <t>Activity statement W1 (blank if not supplied)</t>
-  </si>
-  <si>
-    <t>Expense sign factor</t>
-  </si>
-  <si>
-    <t>Bucket totals (SUMIFS over tblPnl)</t>
-  </si>
-  <si>
-    <t>What the ATO does with it</t>
-  </si>
-  <si>
-    <t>Sales of goods and services. The ATO's turnover label.</t>
-  </si>
-  <si>
-    <t>Business income that is not sales, for example interest or grants.</t>
-  </si>
-  <si>
-    <t>Cost of sales, excluding any salary and wages inside it.</t>
-  </si>
-  <si>
-    <t>Salary and wages included in cost of sales.</t>
-  </si>
-  <si>
-    <t>Salary and wages outside cost of sales.</t>
-  </si>
-  <si>
-    <t>Contractor, subcontractor and commission expenses.</t>
-  </si>
-  <si>
-    <t>Payments to associated persons.</t>
-  </si>
-  <si>
-    <t>Rent expenses.</t>
-  </si>
-  <si>
-    <t>Motor vehicle expenses.</t>
-  </si>
-  <si>
-    <t>Every other expense, including superannuation and depreciation.</t>
-  </si>
-  <si>
-    <t>Not part of the ATO calculation, for example income tax expense.</t>
-  </si>
-  <si>
-    <t>Figures</t>
-  </si>
-  <si>
-    <t>Sales of goods and services</t>
-  </si>
-  <si>
-    <t>Other business income</t>
-  </si>
-  <si>
-    <t>Total business income</t>
-  </si>
-  <si>
-    <t>Turnover</t>
-  </si>
-  <si>
-    <t>Turnover basis</t>
-  </si>
-  <si>
-    <t>Total expenses reported</t>
-  </si>
-  <si>
-    <t>Payments to associated persons</t>
-  </si>
-  <si>
-    <t>Total expenses for ratio</t>
-  </si>
-  <si>
-    <t>Cost of sales for ratio (excludes wages)</t>
-  </si>
-  <si>
-    <t>Salary and wages label (wages + cost of sales wages + associates)</t>
-  </si>
-  <si>
-    <t>Labour base (W1 when it exceeds the label)</t>
-  </si>
-  <si>
-    <t>Labour (base less associates plus contractors and commission)</t>
-  </si>
-  <si>
-    <t>Band lookup (1E9 = no match)</t>
-  </si>
-  <si>
-    <t>Band row in tblBands (0 = none)</t>
-  </si>
-  <si>
-    <t>Turnover band</t>
-  </si>
-  <si>
-    <t>Industry row in tblBands (0 = not published for the year)</t>
-  </si>
-  <si>
-    <t>Published key ratio</t>
-  </si>
-  <si>
-    <t>Key ratio used</t>
-  </si>
-  <si>
-    <t>Ratio</t>
-  </si>
-  <si>
-    <t>Actual</t>
-  </si>
-  <si>
-    <t>Benchmark min</t>
-  </si>
-  <si>
-    <t>Benchmark max</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Range source</t>
-  </si>
-  <si>
-    <t>Cost of sales to turnover</t>
-  </si>
-  <si>
-    <t>Total expenses to turnover</t>
-  </si>
-  <si>
-    <t>labour_to_turnover</t>
-  </si>
-  <si>
-    <t>Labour to turnover</t>
   </si>
   <si>
     <t>Rent to turnover</t>
@@ -21288,11 +21285,17 @@
       <c r="R391">
         <v>0.15</v>
       </c>
+      <c r="S391">
+        <v>0.01</v>
+      </c>
+      <c r="T391">
+        <v>0.03</v>
+      </c>
       <c r="U391" t="s">
+        <v>338</v>
+      </c>
+      <c r="V391" t="s">
         <v>370</v>
-      </c>
-      <c r="V391" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="392" spans="1:22" x14ac:dyDescent="0.25">
@@ -21344,11 +21347,17 @@
       <c r="R392">
         <v>0.1</v>
       </c>
+      <c r="S392">
+        <v>0.01</v>
+      </c>
+      <c r="T392">
+        <v>0.01</v>
+      </c>
       <c r="U392" t="s">
+        <v>338</v>
+      </c>
+      <c r="V392" t="s">
         <v>370</v>
-      </c>
-      <c r="V392" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="393" spans="1:22" x14ac:dyDescent="0.25">
@@ -21397,11 +21406,17 @@
       <c r="R393">
         <v>7.0000000000000007E-2</v>
       </c>
+      <c r="S393">
+        <v>0</v>
+      </c>
+      <c r="T393">
+        <v>0.01</v>
+      </c>
       <c r="U393" t="s">
+        <v>338</v>
+      </c>
+      <c r="V393" t="s">
         <v>370</v>
-      </c>
-      <c r="V393" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="394" spans="1:22" x14ac:dyDescent="0.25">
@@ -21463,7 +21478,7 @@
         <v>335</v>
       </c>
       <c r="V394" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="395" spans="1:22" x14ac:dyDescent="0.25">
@@ -21525,7 +21540,7 @@
         <v>335</v>
       </c>
       <c r="V395" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="396" spans="1:22" x14ac:dyDescent="0.25">
@@ -21584,7 +21599,7 @@
         <v>335</v>
       </c>
       <c r="V396" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="397" spans="1:22" x14ac:dyDescent="0.25">
@@ -21646,7 +21661,7 @@
         <v>330</v>
       </c>
       <c r="V397" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="398" spans="1:22" x14ac:dyDescent="0.25">
@@ -21708,7 +21723,7 @@
         <v>330</v>
       </c>
       <c r="V398" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="399" spans="1:22" x14ac:dyDescent="0.25">
@@ -21767,7 +21782,7 @@
         <v>330</v>
       </c>
       <c r="V399" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="400" spans="1:22" x14ac:dyDescent="0.25">
@@ -21817,7 +21832,7 @@
         <v>343</v>
       </c>
       <c r="V400" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="401" spans="1:22" x14ac:dyDescent="0.25">
@@ -21867,7 +21882,7 @@
         <v>343</v>
       </c>
       <c r="V401" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="402" spans="1:22" x14ac:dyDescent="0.25">
@@ -21914,7 +21929,7 @@
         <v>343</v>
       </c>
       <c r="V402" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="403" spans="1:22" x14ac:dyDescent="0.25">
@@ -21976,7 +21991,7 @@
         <v>335</v>
       </c>
       <c r="V403" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="404" spans="1:22" x14ac:dyDescent="0.25">
@@ -22038,7 +22053,7 @@
         <v>335</v>
       </c>
       <c r="V404" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="405" spans="1:22" x14ac:dyDescent="0.25">
@@ -22097,7 +22112,7 @@
         <v>335</v>
       </c>
       <c r="V405" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="406" spans="1:22" x14ac:dyDescent="0.25">
@@ -22156,10 +22171,10 @@
         <v>0.1</v>
       </c>
       <c r="U406" t="s">
+        <v>375</v>
+      </c>
+      <c r="V406" t="s">
         <v>376</v>
-      </c>
-      <c r="V406" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="407" spans="1:22" x14ac:dyDescent="0.25">
@@ -22218,10 +22233,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="U407" t="s">
+        <v>375</v>
+      </c>
+      <c r="V407" t="s">
         <v>376</v>
-      </c>
-      <c r="V407" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="408" spans="1:22" x14ac:dyDescent="0.25">
@@ -22277,10 +22292,10 @@
         <v>0.04</v>
       </c>
       <c r="U408" t="s">
+        <v>375</v>
+      </c>
+      <c r="V408" t="s">
         <v>376</v>
-      </c>
-      <c r="V408" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="409" spans="1:22" x14ac:dyDescent="0.25">
@@ -22332,11 +22347,17 @@
       <c r="R409">
         <v>0.13</v>
       </c>
+      <c r="S409">
+        <v>0.03</v>
+      </c>
+      <c r="T409">
+        <v>0.05</v>
+      </c>
       <c r="U409" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
       <c r="V409" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="410" spans="1:22" x14ac:dyDescent="0.25">
@@ -22385,11 +22406,17 @@
       <c r="R410">
         <v>0.08</v>
       </c>
+      <c r="S410">
+        <v>0.01</v>
+      </c>
+      <c r="T410">
+        <v>0.01</v>
+      </c>
       <c r="U410" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
       <c r="V410" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="411" spans="1:22" x14ac:dyDescent="0.25">
@@ -22448,10 +22475,10 @@
         <v>0.09</v>
       </c>
       <c r="U411" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V411" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="412" spans="1:22" x14ac:dyDescent="0.25">
@@ -22510,10 +22537,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="U412" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V412" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="413" spans="1:22" x14ac:dyDescent="0.25">
@@ -22569,10 +22596,10 @@
         <v>0.05</v>
       </c>
       <c r="U413" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V413" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="414" spans="1:22" x14ac:dyDescent="0.25">
@@ -22634,7 +22661,7 @@
         <v>335</v>
       </c>
       <c r="V414" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="415" spans="1:22" x14ac:dyDescent="0.25">
@@ -22696,7 +22723,7 @@
         <v>335</v>
       </c>
       <c r="V415" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="416" spans="1:22" x14ac:dyDescent="0.25">
@@ -22755,7 +22782,7 @@
         <v>335</v>
       </c>
       <c r="V416" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="417" spans="1:22" x14ac:dyDescent="0.25">
@@ -22817,7 +22844,7 @@
         <v>335</v>
       </c>
       <c r="V417" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="418" spans="1:22" x14ac:dyDescent="0.25">
@@ -22879,7 +22906,7 @@
         <v>335</v>
       </c>
       <c r="V418" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="419" spans="1:22" x14ac:dyDescent="0.25">
@@ -22938,7 +22965,7 @@
         <v>335</v>
       </c>
       <c r="V419" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="420" spans="1:22" x14ac:dyDescent="0.25">
@@ -23000,7 +23027,7 @@
         <v>335</v>
       </c>
       <c r="V420" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="421" spans="1:22" x14ac:dyDescent="0.25">
@@ -23062,7 +23089,7 @@
         <v>335</v>
       </c>
       <c r="V421" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="422" spans="1:22" x14ac:dyDescent="0.25">
@@ -23121,7 +23148,7 @@
         <v>335</v>
       </c>
       <c r="V422" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="423" spans="1:22" x14ac:dyDescent="0.25">
@@ -23189,7 +23216,7 @@
         <v>338</v>
       </c>
       <c r="V423" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="424" spans="1:22" x14ac:dyDescent="0.25">
@@ -23257,7 +23284,7 @@
         <v>338</v>
       </c>
       <c r="V424" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="425" spans="1:22" x14ac:dyDescent="0.25">
@@ -23322,7 +23349,7 @@
         <v>338</v>
       </c>
       <c r="V425" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="426" spans="1:22" x14ac:dyDescent="0.25">
@@ -23384,7 +23411,7 @@
         <v>335</v>
       </c>
       <c r="V426" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="427" spans="1:22" x14ac:dyDescent="0.25">
@@ -23446,7 +23473,7 @@
         <v>335</v>
       </c>
       <c r="V427" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="428" spans="1:22" x14ac:dyDescent="0.25">
@@ -23505,7 +23532,7 @@
         <v>335</v>
       </c>
       <c r="V428" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="429" spans="1:22" x14ac:dyDescent="0.25">
@@ -23573,7 +23600,7 @@
         <v>338</v>
       </c>
       <c r="V429" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="430" spans="1:22" x14ac:dyDescent="0.25">
@@ -23641,7 +23668,7 @@
         <v>338</v>
       </c>
       <c r="V430" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="431" spans="1:22" x14ac:dyDescent="0.25">
@@ -23706,7 +23733,7 @@
         <v>338</v>
       </c>
       <c r="V431" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="432" spans="1:22" x14ac:dyDescent="0.25">
@@ -23762,7 +23789,7 @@
         <v>343</v>
       </c>
       <c r="V432" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="433" spans="1:22" x14ac:dyDescent="0.25">
@@ -23818,7 +23845,7 @@
         <v>343</v>
       </c>
       <c r="V433" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="434" spans="1:22" x14ac:dyDescent="0.25">
@@ -23871,7 +23898,7 @@
         <v>343</v>
       </c>
       <c r="V434" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="435" spans="1:22" x14ac:dyDescent="0.25">
@@ -23921,7 +23948,7 @@
         <v>343</v>
       </c>
       <c r="V435" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="436" spans="1:22" x14ac:dyDescent="0.25">
@@ -23971,7 +23998,7 @@
         <v>343</v>
       </c>
       <c r="V436" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="437" spans="1:22" x14ac:dyDescent="0.25">
@@ -24018,7 +24045,7 @@
         <v>343</v>
       </c>
       <c r="V437" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="438" spans="1:22" x14ac:dyDescent="0.25">
@@ -24086,7 +24113,7 @@
         <v>338</v>
       </c>
       <c r="V438" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="439" spans="1:22" x14ac:dyDescent="0.25">
@@ -24154,7 +24181,7 @@
         <v>338</v>
       </c>
       <c r="V439" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="440" spans="1:22" x14ac:dyDescent="0.25">
@@ -24219,7 +24246,7 @@
         <v>338</v>
       </c>
       <c r="V440" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="441" spans="1:22" x14ac:dyDescent="0.25">
@@ -24281,7 +24308,7 @@
         <v>335</v>
       </c>
       <c r="V441" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="442" spans="1:22" x14ac:dyDescent="0.25">
@@ -24343,7 +24370,7 @@
         <v>335</v>
       </c>
       <c r="V442" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="443" spans="1:22" x14ac:dyDescent="0.25">
@@ -24402,7 +24429,7 @@
         <v>335</v>
       </c>
       <c r="V443" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="444" spans="1:22" x14ac:dyDescent="0.25">
@@ -24464,7 +24491,7 @@
         <v>335</v>
       </c>
       <c r="V444" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="445" spans="1:22" x14ac:dyDescent="0.25">
@@ -24526,7 +24553,7 @@
         <v>335</v>
       </c>
       <c r="V445" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="446" spans="1:22" x14ac:dyDescent="0.25">
@@ -24585,7 +24612,7 @@
         <v>335</v>
       </c>
       <c r="V446" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="447" spans="1:22" x14ac:dyDescent="0.25">
@@ -24647,7 +24674,7 @@
         <v>330</v>
       </c>
       <c r="V447" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="448" spans="1:22" x14ac:dyDescent="0.25">
@@ -24709,7 +24736,7 @@
         <v>330</v>
       </c>
       <c r="V448" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="449" spans="1:22" x14ac:dyDescent="0.25">
@@ -24768,7 +24795,7 @@
         <v>330</v>
       </c>
       <c r="V449" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="450" spans="1:22" x14ac:dyDescent="0.25">
@@ -24820,11 +24847,17 @@
       <c r="R450">
         <v>0.15</v>
       </c>
+      <c r="S450">
+        <v>0.02</v>
+      </c>
+      <c r="T450">
+        <v>0.03</v>
+      </c>
       <c r="U450" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
       <c r="V450" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="451" spans="1:22" x14ac:dyDescent="0.25">
@@ -24876,11 +24909,17 @@
       <c r="R451">
         <v>0.11</v>
       </c>
+      <c r="S451">
+        <v>0.01</v>
+      </c>
+      <c r="T451">
+        <v>0.02</v>
+      </c>
       <c r="U451" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
       <c r="V451" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="452" spans="1:22" x14ac:dyDescent="0.25">
@@ -24929,11 +24968,17 @@
       <c r="R452">
         <v>0.06</v>
       </c>
+      <c r="S452">
+        <v>0</v>
+      </c>
+      <c r="T452">
+        <v>0.01</v>
+      </c>
       <c r="U452" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
       <c r="V452" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="453" spans="1:22" x14ac:dyDescent="0.25">
@@ -25001,7 +25046,7 @@
         <v>332</v>
       </c>
       <c r="V453" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="454" spans="1:22" x14ac:dyDescent="0.25">
@@ -25069,7 +25114,7 @@
         <v>332</v>
       </c>
       <c r="V454" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="455" spans="1:22" x14ac:dyDescent="0.25">
@@ -25134,7 +25179,7 @@
         <v>332</v>
       </c>
       <c r="V455" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="456" spans="1:22" x14ac:dyDescent="0.25">
@@ -25325,7 +25370,7 @@
         <v>338</v>
       </c>
       <c r="V459" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="460" spans="1:22" x14ac:dyDescent="0.25">
@@ -25387,7 +25432,7 @@
         <v>338</v>
       </c>
       <c r="V460" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="461" spans="1:22" x14ac:dyDescent="0.25">
@@ -25446,7 +25491,7 @@
         <v>338</v>
       </c>
       <c r="V461" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="462" spans="1:22" x14ac:dyDescent="0.25">
@@ -25508,7 +25553,7 @@
         <v>335</v>
       </c>
       <c r="V462" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="463" spans="1:22" x14ac:dyDescent="0.25">
@@ -25570,7 +25615,7 @@
         <v>335</v>
       </c>
       <c r="V463" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="464" spans="1:22" x14ac:dyDescent="0.25">
@@ -25629,7 +25674,7 @@
         <v>335</v>
       </c>
       <c r="V464" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="465" spans="1:22" x14ac:dyDescent="0.25">
@@ -25697,7 +25742,7 @@
         <v>338</v>
       </c>
       <c r="V465" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="466" spans="1:22" x14ac:dyDescent="0.25">
@@ -25765,7 +25810,7 @@
         <v>338</v>
       </c>
       <c r="V466" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="467" spans="1:22" x14ac:dyDescent="0.25">
@@ -25830,7 +25875,7 @@
         <v>338</v>
       </c>
       <c r="V467" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="468" spans="1:22" x14ac:dyDescent="0.25">
@@ -25892,7 +25937,7 @@
         <v>335</v>
       </c>
       <c r="V468" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="469" spans="1:22" x14ac:dyDescent="0.25">
@@ -25954,7 +25999,7 @@
         <v>335</v>
       </c>
       <c r="V469" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="470" spans="1:22" x14ac:dyDescent="0.25">
@@ -26013,7 +26058,7 @@
         <v>335</v>
       </c>
       <c r="V470" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="471" spans="1:22" x14ac:dyDescent="0.25">
@@ -26075,7 +26120,7 @@
         <v>335</v>
       </c>
       <c r="V471" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="472" spans="1:22" x14ac:dyDescent="0.25">
@@ -26137,7 +26182,7 @@
         <v>335</v>
       </c>
       <c r="V472" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="473" spans="1:22" x14ac:dyDescent="0.25">
@@ -26196,7 +26241,7 @@
         <v>335</v>
       </c>
       <c r="V473" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="474" spans="1:22" x14ac:dyDescent="0.25">
@@ -26255,10 +26300,10 @@
         <v>0.11</v>
       </c>
       <c r="U474" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V474" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="475" spans="1:22" x14ac:dyDescent="0.25">
@@ -26317,10 +26362,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="U475" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V475" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="476" spans="1:22" x14ac:dyDescent="0.25">
@@ -26376,10 +26421,10 @@
         <v>0.05</v>
       </c>
       <c r="U476" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V476" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="477" spans="1:22" x14ac:dyDescent="0.25">
@@ -26435,7 +26480,7 @@
         <v>335</v>
       </c>
       <c r="V477" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="478" spans="1:22" x14ac:dyDescent="0.25">
@@ -26491,7 +26536,7 @@
         <v>335</v>
       </c>
       <c r="V478" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="479" spans="1:22" x14ac:dyDescent="0.25">
@@ -26544,7 +26589,7 @@
         <v>335</v>
       </c>
       <c r="V479" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="480" spans="1:22" x14ac:dyDescent="0.25">
@@ -26600,7 +26645,7 @@
         <v>343</v>
       </c>
       <c r="V480" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="481" spans="1:22" x14ac:dyDescent="0.25">
@@ -26656,7 +26701,7 @@
         <v>343</v>
       </c>
       <c r="V481" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="482" spans="1:22" x14ac:dyDescent="0.25">
@@ -26709,7 +26754,7 @@
         <v>343</v>
       </c>
       <c r="V482" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="483" spans="1:22" x14ac:dyDescent="0.25">
@@ -26765,7 +26810,7 @@
         <v>347</v>
       </c>
       <c r="V483" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="484" spans="1:22" x14ac:dyDescent="0.25">
@@ -26821,7 +26866,7 @@
         <v>347</v>
       </c>
       <c r="V484" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="485" spans="1:22" x14ac:dyDescent="0.25">
@@ -26874,7 +26919,7 @@
         <v>347</v>
       </c>
       <c r="V485" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="486" spans="1:22" x14ac:dyDescent="0.25">
@@ -26942,7 +26987,7 @@
         <v>332</v>
       </c>
       <c r="V486" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="487" spans="1:22" x14ac:dyDescent="0.25">
@@ -27010,7 +27055,7 @@
         <v>332</v>
       </c>
       <c r="V487" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="488" spans="1:22" x14ac:dyDescent="0.25">
@@ -27075,7 +27120,7 @@
         <v>332</v>
       </c>
       <c r="V488" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="489" spans="1:22" x14ac:dyDescent="0.25">
@@ -27137,7 +27182,7 @@
         <v>335</v>
       </c>
       <c r="V489" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="490" spans="1:22" x14ac:dyDescent="0.25">
@@ -27199,7 +27244,7 @@
         <v>335</v>
       </c>
       <c r="V490" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="491" spans="1:22" x14ac:dyDescent="0.25">
@@ -27258,7 +27303,7 @@
         <v>335</v>
       </c>
       <c r="V491" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="492" spans="1:22" x14ac:dyDescent="0.25">
@@ -27320,7 +27365,7 @@
         <v>335</v>
       </c>
       <c r="V492" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="493" spans="1:22" x14ac:dyDescent="0.25">
@@ -27382,7 +27427,7 @@
         <v>335</v>
       </c>
       <c r="V493" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="494" spans="1:22" x14ac:dyDescent="0.25">
@@ -27441,7 +27486,7 @@
         <v>335</v>
       </c>
       <c r="V494" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="495" spans="1:22" x14ac:dyDescent="0.25">
@@ -27509,7 +27554,7 @@
         <v>338</v>
       </c>
       <c r="V495" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="496" spans="1:22" x14ac:dyDescent="0.25">
@@ -27577,7 +27622,7 @@
         <v>338</v>
       </c>
       <c r="V496" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="497" spans="1:22" x14ac:dyDescent="0.25">
@@ -27642,7 +27687,7 @@
         <v>338</v>
       </c>
       <c r="V497" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="498" spans="1:22" x14ac:dyDescent="0.25">
@@ -27704,7 +27749,7 @@
         <v>335</v>
       </c>
       <c r="V498" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="499" spans="1:22" x14ac:dyDescent="0.25">
@@ -27766,7 +27811,7 @@
         <v>335</v>
       </c>
       <c r="V499" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="500" spans="1:22" x14ac:dyDescent="0.25">
@@ -27825,7 +27870,7 @@
         <v>335</v>
       </c>
       <c r="V500" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="501" spans="1:22" x14ac:dyDescent="0.25">
@@ -27887,7 +27932,7 @@
         <v>335</v>
       </c>
       <c r="V501" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="502" spans="1:22" x14ac:dyDescent="0.25">
@@ -27949,7 +27994,7 @@
         <v>335</v>
       </c>
       <c r="V502" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="503" spans="1:22" x14ac:dyDescent="0.25">
@@ -28008,7 +28053,7 @@
         <v>335</v>
       </c>
       <c r="V503" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="504" spans="1:22" x14ac:dyDescent="0.25">
@@ -28070,7 +28115,7 @@
         <v>335</v>
       </c>
       <c r="V504" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="505" spans="1:22" x14ac:dyDescent="0.25">
@@ -28132,7 +28177,7 @@
         <v>335</v>
       </c>
       <c r="V505" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="506" spans="1:22" x14ac:dyDescent="0.25">
@@ -28191,7 +28236,7 @@
         <v>335</v>
       </c>
       <c r="V506" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="507" spans="1:22" x14ac:dyDescent="0.25">
@@ -28250,10 +28295,10 @@
         <v>0.11</v>
       </c>
       <c r="U507" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V507" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="508" spans="1:22" x14ac:dyDescent="0.25">
@@ -28312,10 +28357,10 @@
         <v>0.06</v>
       </c>
       <c r="U508" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V508" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="509" spans="1:22" x14ac:dyDescent="0.25">
@@ -28371,10 +28416,10 @@
         <v>0.04</v>
       </c>
       <c r="U509" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V509" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="510" spans="1:22" x14ac:dyDescent="0.25">
@@ -28442,7 +28487,7 @@
         <v>332</v>
       </c>
       <c r="V510" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="511" spans="1:22" x14ac:dyDescent="0.25">
@@ -28510,7 +28555,7 @@
         <v>332</v>
       </c>
       <c r="V511" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="512" spans="1:22" x14ac:dyDescent="0.25">
@@ -28575,7 +28620,7 @@
         <v>332</v>
       </c>
       <c r="V512" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="513" spans="1:22" x14ac:dyDescent="0.25">
@@ -28631,7 +28676,7 @@
         <v>347</v>
       </c>
       <c r="V513" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="514" spans="1:22" x14ac:dyDescent="0.25">
@@ -28687,7 +28732,7 @@
         <v>347</v>
       </c>
       <c r="V514" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="515" spans="1:22" x14ac:dyDescent="0.25">
@@ -28740,7 +28785,7 @@
         <v>347</v>
       </c>
       <c r="V515" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="516" spans="1:22" x14ac:dyDescent="0.25">
@@ -28802,7 +28847,7 @@
         <v>335</v>
       </c>
       <c r="V516" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="517" spans="1:22" x14ac:dyDescent="0.25">
@@ -28864,7 +28909,7 @@
         <v>335</v>
       </c>
       <c r="V517" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="518" spans="1:22" x14ac:dyDescent="0.25">
@@ -28923,7 +28968,7 @@
         <v>335</v>
       </c>
       <c r="V518" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="519" spans="1:22" x14ac:dyDescent="0.25">
@@ -28991,7 +29036,7 @@
         <v>338</v>
       </c>
       <c r="V519" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="520" spans="1:22" x14ac:dyDescent="0.25">
@@ -29059,7 +29104,7 @@
         <v>338</v>
       </c>
       <c r="V520" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="521" spans="1:22" x14ac:dyDescent="0.25">
@@ -29124,7 +29169,7 @@
         <v>338</v>
       </c>
       <c r="V521" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="522" spans="1:22" x14ac:dyDescent="0.25">
@@ -29186,7 +29231,7 @@
         <v>338</v>
       </c>
       <c r="V522" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="523" spans="1:22" x14ac:dyDescent="0.25">
@@ -29248,7 +29293,7 @@
         <v>338</v>
       </c>
       <c r="V523" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="524" spans="1:22" x14ac:dyDescent="0.25">
@@ -29307,7 +29352,7 @@
         <v>338</v>
       </c>
       <c r="V524" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="525" spans="1:22" x14ac:dyDescent="0.25">
@@ -29369,7 +29414,7 @@
         <v>335</v>
       </c>
       <c r="V525" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="526" spans="1:22" x14ac:dyDescent="0.25">
@@ -29431,7 +29476,7 @@
         <v>335</v>
       </c>
       <c r="V526" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="527" spans="1:22" x14ac:dyDescent="0.25">
@@ -29490,7 +29535,7 @@
         <v>335</v>
       </c>
       <c r="V527" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="528" spans="1:22" x14ac:dyDescent="0.25">
@@ -29552,7 +29597,7 @@
         <v>335</v>
       </c>
       <c r="V528" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="529" spans="1:22" x14ac:dyDescent="0.25">
@@ -29614,7 +29659,7 @@
         <v>335</v>
       </c>
       <c r="V529" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="530" spans="1:22" x14ac:dyDescent="0.25">
@@ -29673,7 +29718,7 @@
         <v>335</v>
       </c>
       <c r="V530" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="531" spans="1:22" x14ac:dyDescent="0.25">
@@ -29732,10 +29777,10 @@
         <v>0.1</v>
       </c>
       <c r="U531" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V531" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="532" spans="1:22" x14ac:dyDescent="0.25">
@@ -29794,10 +29839,10 @@
         <v>0.05</v>
       </c>
       <c r="U532" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V532" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="533" spans="1:22" x14ac:dyDescent="0.25">
@@ -29853,10 +29898,10 @@
         <v>0.02</v>
       </c>
       <c r="U533" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V533" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="534" spans="1:22" x14ac:dyDescent="0.25">
@@ -29915,10 +29960,10 @@
         <v>0.11</v>
       </c>
       <c r="U534" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V534" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="535" spans="1:22" x14ac:dyDescent="0.25">
@@ -29977,10 +30022,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="U535" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V535" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="536" spans="1:22" x14ac:dyDescent="0.25">
@@ -30036,10 +30081,10 @@
         <v>0.05</v>
       </c>
       <c r="U536" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="V536" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="537" spans="1:22" x14ac:dyDescent="0.25">
@@ -30107,7 +30152,7 @@
         <v>338</v>
       </c>
       <c r="V537" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="538" spans="1:22" x14ac:dyDescent="0.25">
@@ -30175,7 +30220,7 @@
         <v>338</v>
       </c>
       <c r="V538" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="539" spans="1:22" x14ac:dyDescent="0.25">
@@ -30240,7 +30285,7 @@
         <v>338</v>
       </c>
       <c r="V539" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="540" spans="1:22" x14ac:dyDescent="0.25">
@@ -30286,11 +30331,29 @@
       <c r="N540" t="s">
         <v>329</v>
       </c>
+      <c r="O540">
+        <v>0.19</v>
+      </c>
+      <c r="P540">
+        <v>0.3</v>
+      </c>
+      <c r="Q540">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="R540">
+        <v>0.13</v>
+      </c>
+      <c r="S540">
+        <v>0.04</v>
+      </c>
+      <c r="T540">
+        <v>0.06</v>
+      </c>
       <c r="U540" t="s">
-        <v>116</v>
+        <v>332</v>
       </c>
       <c r="V540" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="541" spans="1:22" x14ac:dyDescent="0.25">
@@ -30336,11 +30399,29 @@
       <c r="N541" t="s">
         <v>329</v>
       </c>
+      <c r="O541">
+        <v>0.16</v>
+      </c>
+      <c r="P541">
+        <v>0.27</v>
+      </c>
+      <c r="Q541">
+        <v>0.06</v>
+      </c>
+      <c r="R541">
+        <v>0.09</v>
+      </c>
+      <c r="S541">
+        <v>0.02</v>
+      </c>
+      <c r="T541">
+        <v>0.03</v>
+      </c>
       <c r="U541" t="s">
-        <v>116</v>
+        <v>332</v>
       </c>
       <c r="V541" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="542" spans="1:22" x14ac:dyDescent="0.25">
@@ -30383,11 +30464,29 @@
       <c r="N542" t="s">
         <v>329</v>
       </c>
+      <c r="O542">
+        <v>0.18</v>
+      </c>
+      <c r="P542">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="Q542">
+        <v>0.04</v>
+      </c>
+      <c r="R542">
+        <v>0.06</v>
+      </c>
+      <c r="S542">
+        <v>0.01</v>
+      </c>
+      <c r="T542">
+        <v>0.02</v>
+      </c>
       <c r="U542" t="s">
-        <v>116</v>
+        <v>332</v>
       </c>
       <c r="V542" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="543" spans="1:22" x14ac:dyDescent="0.25">
@@ -30455,7 +30554,7 @@
         <v>338</v>
       </c>
       <c r="V543" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="544" spans="1:22" x14ac:dyDescent="0.25">
@@ -30523,7 +30622,7 @@
         <v>338</v>
       </c>
       <c r="V544" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="545" spans="1:22" x14ac:dyDescent="0.25">
@@ -30588,7 +30687,7 @@
         <v>338</v>
       </c>
       <c r="V545" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="546" spans="1:22" x14ac:dyDescent="0.25">
@@ -30656,7 +30755,7 @@
         <v>338</v>
       </c>
       <c r="V546" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="547" spans="1:22" x14ac:dyDescent="0.25">
@@ -30724,7 +30823,7 @@
         <v>338</v>
       </c>
       <c r="V547" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="548" spans="1:22" x14ac:dyDescent="0.25">
@@ -30789,7 +30888,7 @@
         <v>338</v>
       </c>
       <c r="V548" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="549" spans="1:22" x14ac:dyDescent="0.25">
@@ -30845,7 +30944,7 @@
         <v>347</v>
       </c>
       <c r="V549" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="550" spans="1:22" x14ac:dyDescent="0.25">
@@ -30901,7 +31000,7 @@
         <v>347</v>
       </c>
       <c r="V550" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="551" spans="1:22" x14ac:dyDescent="0.25">
@@ -30954,7 +31053,7 @@
         <v>347</v>
       </c>
       <c r="V551" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="552" spans="1:22" x14ac:dyDescent="0.25">
@@ -31010,7 +31109,7 @@
         <v>347</v>
       </c>
       <c r="V552" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="553" spans="1:22" x14ac:dyDescent="0.25">
@@ -31066,7 +31165,7 @@
         <v>347</v>
       </c>
       <c r="V553" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="554" spans="1:22" x14ac:dyDescent="0.25">
@@ -31119,7 +31218,7 @@
         <v>347</v>
       </c>
       <c r="V554" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="555" spans="1:22" x14ac:dyDescent="0.25">
@@ -31175,7 +31274,7 @@
         <v>335</v>
       </c>
       <c r="V555" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="556" spans="1:22" x14ac:dyDescent="0.25">
@@ -31231,7 +31330,7 @@
         <v>335</v>
       </c>
       <c r="V556" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="557" spans="1:22" x14ac:dyDescent="0.25">
@@ -31284,7 +31383,7 @@
         <v>335</v>
       </c>
       <c r="V557" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="558" spans="1:22" x14ac:dyDescent="0.25">
@@ -31352,7 +31451,7 @@
         <v>338</v>
       </c>
       <c r="V558" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="559" spans="1:22" x14ac:dyDescent="0.25">
@@ -31420,7 +31519,7 @@
         <v>338</v>
       </c>
       <c r="V559" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="560" spans="1:22" x14ac:dyDescent="0.25">
@@ -31485,7 +31584,7 @@
         <v>338</v>
       </c>
       <c r="V560" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="561" spans="1:22" x14ac:dyDescent="0.25">
@@ -31547,7 +31646,7 @@
         <v>335</v>
       </c>
       <c r="V561" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="562" spans="1:22" x14ac:dyDescent="0.25">
@@ -31609,7 +31708,7 @@
         <v>335</v>
       </c>
       <c r="V562" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="563" spans="1:22" x14ac:dyDescent="0.25">
@@ -31668,7 +31767,7 @@
         <v>335</v>
       </c>
       <c r="V563" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="564" spans="1:22" x14ac:dyDescent="0.25">
@@ -31736,7 +31835,7 @@
         <v>338</v>
       </c>
       <c r="V564" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="565" spans="1:22" x14ac:dyDescent="0.25">
@@ -31804,7 +31903,7 @@
         <v>338</v>
       </c>
       <c r="V565" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="566" spans="1:22" x14ac:dyDescent="0.25">
@@ -31869,7 +31968,7 @@
         <v>338</v>
       </c>
       <c r="V566" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="567" spans="1:22" x14ac:dyDescent="0.25">
@@ -31922,10 +32021,10 @@
         <v>0.11</v>
       </c>
       <c r="U567" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="V567" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="568" spans="1:22" x14ac:dyDescent="0.25">
@@ -31978,10 +32077,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="U568" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="V568" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="569" spans="1:22" x14ac:dyDescent="0.25">
@@ -32031,10 +32130,10 @@
         <v>0.03</v>
       </c>
       <c r="U569" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="V569" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="570" spans="1:22" x14ac:dyDescent="0.25">
@@ -32087,10 +32186,10 @@
         <v>0.12</v>
       </c>
       <c r="U570" t="s">
+        <v>429</v>
+      </c>
+      <c r="V570" t="s">
         <v>431</v>
-      </c>
-      <c r="V570" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="571" spans="1:22" x14ac:dyDescent="0.25">
@@ -32143,10 +32242,10 @@
         <v>0.09</v>
       </c>
       <c r="U571" t="s">
+        <v>429</v>
+      </c>
+      <c r="V571" t="s">
         <v>431</v>
-      </c>
-      <c r="V571" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="572" spans="1:22" x14ac:dyDescent="0.25">
@@ -32196,10 +32295,10 @@
         <v>0.06</v>
       </c>
       <c r="U572" t="s">
+        <v>429</v>
+      </c>
+      <c r="V572" t="s">
         <v>431</v>
-      </c>
-      <c r="V572" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="573" spans="1:22" x14ac:dyDescent="0.25">
@@ -32261,7 +32360,7 @@
         <v>335</v>
       </c>
       <c r="V573" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="574" spans="1:22" x14ac:dyDescent="0.25">
@@ -32323,7 +32422,7 @@
         <v>335</v>
       </c>
       <c r="V574" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="575" spans="1:22" x14ac:dyDescent="0.25">
@@ -32382,7 +32481,7 @@
         <v>335</v>
       </c>
       <c r="V575" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="576" spans="1:22" x14ac:dyDescent="0.25">
@@ -32444,7 +32543,7 @@
         <v>338</v>
       </c>
       <c r="V576" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="577" spans="1:22" x14ac:dyDescent="0.25">
@@ -32506,7 +32605,7 @@
         <v>338</v>
       </c>
       <c r="V577" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="578" spans="1:22" x14ac:dyDescent="0.25">
@@ -32565,7 +32664,7 @@
         <v>338</v>
       </c>
       <c r="V578" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="579" spans="1:22" x14ac:dyDescent="0.25">
@@ -32627,7 +32726,7 @@
         <v>335</v>
       </c>
       <c r="V579" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="580" spans="1:22" x14ac:dyDescent="0.25">
@@ -32689,7 +32788,7 @@
         <v>335</v>
       </c>
       <c r="V580" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="581" spans="1:22" x14ac:dyDescent="0.25">
@@ -32748,7 +32847,7 @@
         <v>335</v>
       </c>
       <c r="V581" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="582" spans="1:22" x14ac:dyDescent="0.25">
@@ -32810,7 +32909,7 @@
         <v>338</v>
       </c>
       <c r="V582" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="583" spans="1:22" x14ac:dyDescent="0.25">
@@ -32872,7 +32971,7 @@
         <v>338</v>
       </c>
       <c r="V583" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="584" spans="1:22" x14ac:dyDescent="0.25">
@@ -32931,7 +33030,7 @@
         <v>338</v>
       </c>
       <c r="V584" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="585" spans="1:22" x14ac:dyDescent="0.25">
@@ -32999,7 +33098,7 @@
         <v>338</v>
       </c>
       <c r="V585" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="586" spans="1:22" x14ac:dyDescent="0.25">
@@ -33067,7 +33166,7 @@
         <v>338</v>
       </c>
       <c r="V586" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="587" spans="1:22" x14ac:dyDescent="0.25">
@@ -33132,7 +33231,7 @@
         <v>338</v>
       </c>
       <c r="V587" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="588" spans="1:22" x14ac:dyDescent="0.25">
@@ -33194,7 +33293,7 @@
         <v>330</v>
       </c>
       <c r="V588" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="589" spans="1:22" x14ac:dyDescent="0.25">
@@ -33256,7 +33355,7 @@
         <v>330</v>
       </c>
       <c r="V589" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="590" spans="1:22" x14ac:dyDescent="0.25">
@@ -33315,7 +33414,7 @@
         <v>330</v>
       </c>
       <c r="V590" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="591" spans="1:22" x14ac:dyDescent="0.25">
@@ -33383,7 +33482,7 @@
         <v>338</v>
       </c>
       <c r="V591" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="592" spans="1:22" x14ac:dyDescent="0.25">
@@ -33451,7 +33550,7 @@
         <v>338</v>
       </c>
       <c r="V592" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="593" spans="1:22" x14ac:dyDescent="0.25">
@@ -33516,7 +33615,7 @@
         <v>338</v>
       </c>
       <c r="V593" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>
@@ -33540,13 +33639,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>328</v>
@@ -33562,7 +33661,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>102</v>
@@ -33570,13 +33669,13 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B6">
         <f>IF(B4="Y",-1,1)</f>
@@ -33585,11 +33684,11 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -33601,7 +33700,7 @@
         <v>850000</v>
       </c>
       <c r="C8" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -33613,7 +33712,7 @@
         <v>1200</v>
       </c>
       <c r="C9" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -33625,7 +33724,7 @@
         <v>270000</v>
       </c>
       <c r="C10" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -33637,7 +33736,7 @@
         <v>95000</v>
       </c>
       <c r="C11" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -33649,7 +33748,7 @@
         <v>175000</v>
       </c>
       <c r="C12" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -33661,7 +33760,7 @@
         <v>7800</v>
       </c>
       <c r="C13" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -33673,7 +33772,7 @@
         <v>45000</v>
       </c>
       <c r="C14" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -33685,7 +33784,7 @@
         <v>62000</v>
       </c>
       <c r="C15" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -33697,7 +33796,7 @@
         <v>9500</v>
       </c>
       <c r="C16" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -33709,7 +33808,7 @@
         <v>87650</v>
       </c>
       <c r="C17" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -33721,18 +33820,18 @@
         <v>2287850</v>
       </c>
       <c r="C18" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B19" s="5"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B20" s="12">
         <f>B8</f>
@@ -33741,7 +33840,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="B21" s="12">
         <f>B9</f>
@@ -33750,7 +33849,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B22" s="12">
         <f>B20+B21</f>
@@ -33759,7 +33858,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B23" s="12">
         <f>IF(OR(B20&lt;=0,B20*2&lt;B22),B22,B20)</f>
@@ -33768,7 +33867,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B24" s="12" t="str">
         <f>IF(OR(B20&lt;=0,B20*2&lt;B22),"total business income","sales of goods and services")</f>
@@ -33777,7 +33876,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B25" s="12">
         <f>SUM(B10:B17)</f>
@@ -33786,7 +33885,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B26" s="12">
         <f>B14</f>
@@ -33795,7 +33894,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B27" s="12">
         <f>B25-B26</f>
@@ -33804,7 +33903,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B28" s="12">
         <f>B10</f>
@@ -33813,7 +33912,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B29" s="12">
         <f>B12+B11+B26</f>
@@ -33822,7 +33921,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B30" s="12">
         <f>IF(AND(B5&lt;&gt;"",B5&gt;B29),B5,B29)</f>
@@ -33831,7 +33930,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B31" s="12">
         <f>B30-B26+B13</f>
@@ -33840,7 +33939,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B32" s="8">
         <f>SUMPRODUCT(MIN(((tblBands[Year]=B2)*(tblBands[Industry]=B3)*(((B23&gt;tblBands[From])+((tblBands[FromInclusive]="Y")*(B23=tblBands[From])))&gt;0)*(((tblBands[To]="")+(B23&lt;=tblBands[To]))&gt;0))*(ROW(tblBands[Year])-1)+(1-((tblBands[Year]=B2)*(tblBands[Industry]=B3)*(((B23&gt;tblBands[From])+((tblBands[FromInclusive]="Y")*(B23=tblBands[From])))&gt;0)*(((tblBands[To]="")+(B23&lt;=tblBands[To]))&gt;0)))*1000000000))</f>
@@ -33849,7 +33948,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B33" s="8">
         <f>IF(B32&gt;=1000000000,0,B32)</f>
@@ -33858,7 +33957,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B34" s="8" t="str">
         <f>IF(B33=0,"none applies",INDEX(tblBands[Label],B33))</f>
@@ -33867,7 +33966,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B35" s="8">
         <f>SUMPRODUCT(MAX((tblBands[Year]=B2)*(tblBands[Industry]=B3)*(ROW(tblBands[Year])-1)))</f>
@@ -33876,7 +33975,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B36" s="8" t="str">
         <f>IF(B35=0,"",INDEX(tblBands[KeyRatio],B35))</f>
@@ -33885,7 +33984,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B37" s="8" t="str">
         <f>IF(AND(B36="cost_of_sales_to_turnover",B28=0),"total_expenses_to_turnover",B36)</f>
@@ -33934,28 +34033,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>479</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>481</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>482</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -33963,7 +34062,7 @@
         <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C2" s="13">
         <f>IFERROR(ROUND(Calculation!B28/Calculation!B23,4),"")</f>
@@ -33995,7 +34094,7 @@
         <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C3" s="13">
         <f>IFERROR(ROUND(Calculation!B27/Calculation!B23,4),"")</f>
@@ -34024,10 +34123,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B4" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C4" s="13">
         <f>IFERROR(ROUND(Calculation!B31/Calculation!B23,4),"")</f>
@@ -34056,10 +34155,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>378</v>
+        <v>486</v>
       </c>
       <c r="B5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C5" s="13">
         <f>IFERROR(ROUND(Calculation!B15/Calculation!B23,4),"")</f>
@@ -34091,7 +34190,7 @@
         <v>343</v>
       </c>
       <c r="B6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C6" s="13">
         <f>IFERROR(ROUND(Calculation!B16/Calculation!B23,4),"")</f>
@@ -34120,7 +34219,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B8" s="12">
         <f>Calculation!B23</f>
@@ -34129,7 +34228,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B9" s="8" t="str">
         <f>Calculation!B34</f>
@@ -34138,7 +34237,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B10" s="8" t="str">
         <f>Calculation!B2&amp;" "&amp;Calculation!B3</f>
@@ -34164,21 +34263,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>491</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>492</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>493</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B2" s="8" t="str">
         <f>IF(C2=0,"PASS","BLOCKED")</f>
@@ -34195,7 +34294,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B3" s="8" t="str">
         <f>IF(C3=0,"PASS","BLOCKED")</f>
@@ -34212,7 +34311,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B4" s="8" t="str">
         <f>IF(C4=0,"PASS","BLOCKED")</f>
@@ -34229,7 +34328,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B5" s="8" t="str">
         <f>IF(C5=0,"PASS","BLOCKED")</f>
@@ -34246,7 +34345,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B6" s="8" t="str">
         <f>IF(C6=0,"PASS","BLOCKED")</f>
@@ -34263,7 +34362,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B7" s="8" t="str">
         <f>IF(AND(Calculation!B5&lt;&gt;"",Calculation!B5&lt;0),"BLOCKED","PASS")</f>
@@ -34277,7 +34376,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B8" s="8" t="str">
         <f>IF(Calculation!B23&gt;0,"PASS","BLOCKED")</f>
@@ -34291,7 +34390,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B9" s="8" t="str">
         <f>IF(Calculation!B35=0,"BLOCKED","PASS")</f>
@@ -34305,7 +34404,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B10" s="8" t="str">
         <f>IF(Calculation!B33=0,"REVIEW","PASS")</f>
@@ -34319,7 +34418,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B11" s="8" t="str">
         <f>IF(C11="within","PASS","REVIEW")</f>
@@ -34333,7 +34432,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B12" s="8" t="str">
         <f>IF(C12=0,"PASS","REVIEW")</f>
@@ -34359,7 +34458,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -34438,55 +34537,55 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>507</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B2" t="s">
         <v>509</v>
-      </c>
-      <c r="B2" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>511</v>
+      </c>
+      <c r="B4" t="s">
         <v>512</v>
-      </c>
-      <c r="B4" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B5" t="s">
         <v>514</v>
-      </c>
-      <c r="B5" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>515</v>
+      </c>
+      <c r="B6" t="s">
         <v>516</v>
-      </c>
-      <c r="B6" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B7" t="s">
         <v>98</v>
@@ -34494,7 +34593,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B8" t="s">
         <v>99</v>
@@ -34502,39 +34601,39 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>519</v>
+      </c>
+      <c r="B9" t="s">
         <v>520</v>
-      </c>
-      <c r="B9" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B10" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B11" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>523</v>
+      </c>
+      <c r="B12" t="s">
         <v>524</v>
-      </c>
-      <c r="B12" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B13" t="s">
         <v>98</v>
@@ -34542,7 +34641,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B14" t="s">
         <v>329</v>
@@ -34550,50 +34649,50 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B15" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>528</v>
+      </c>
+      <c r="B16" t="s">
         <v>529</v>
-      </c>
-      <c r="B16" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>530</v>
+      </c>
+      <c r="B17" t="s">
         <v>531</v>
-      </c>
-      <c r="B17" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>532</v>
+      </c>
+      <c r="B18" t="s">
         <v>533</v>
-      </c>
-      <c r="B18" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>534</v>
+      </c>
+      <c r="B19" t="s">
         <v>535</v>
-      </c>
-      <c r="B19" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>536</v>
+      </c>
+      <c r="B20" t="s">
         <v>537</v>
-      </c>
-      <c r="B20" t="s">
-        <v>538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release ato-benchmark-compare 0.1.11 (#321)
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903EECC8-0800-4006-B205-13B4FD7BFAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD96C1C7-EC53-4EBD-A353-00B4B2CE086C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.1.10. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.1.11. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1567,7 +1567,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.10</t>
+    <t>0.1.11</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Prepare five engine releases: the-exchequer-tally 0.1.8, payday-super-checker 0.1.10, the-wip-tally 0.1.4, australian-tax-calculators 0.1.9 and ato-benchmark-compare 0.1.12
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD96C1C7-EC53-4EBD-A353-00B4B2CE086C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B613EA8-7F6D-4312-BBED-9B985C9BD812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.1.11. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.1.12. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1567,7 +1567,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.11</t>
+    <t>0.1.12</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -1654,7 +1654,7 @@
     <t>Not all expenses are reported by every business. The ATO says to use these ranges only as a guide where they apply to the business.</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20430</t>
+    <t>Excel 16.0 build 20527</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Cut patch releases for the four engines whose release runs failed
payday-super-checker 0.2.0, solomons-sword 0.3.0, ato-benchmark-compare
0.2.0 and div7a-loan-review 0.3.0 were tagged but never released: their
release runs stopped at the test gate because the fast-check worker was
not installed, which #419 fixes. Release the same changes as
payday-super-checker 0.2.1, solomons-sword 0.3.1, ato-benchmark-compare
0.2.1 and div7a-loan-review 0.3.1, and record the unreleased versions in
each release note.

The three workbooks are rebuilt with the desktop Excel pass and differ
only in their two version cells. The MCP's div7a test and quick-proof
transcript follow the workspace engine to 0.3.1.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BDC12F1-D8FC-4D88-83EC-17F5D50B7CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CCB8D2-AD7F-4507-A3D7-AE94E5591817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.2.0. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.2.1. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1567,7 +1567,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.2.1</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Cut 0.2.2 and 0.3.2 for the four engines after the 0.2.1 runs stopped
The payday-super-checker 0.2.1, solomons-sword 0.3.1,
ato-benchmark-compare 0.2.1 and div7a-loan-review 0.3.1 release runs
passed their tests, then stopped at the publish gate because main moved
while they ran. Nothing was published. Release the same changes as
payday-super-checker 0.2.2, solomons-sword 0.3.2, ato-benchmark-compare
0.2.2 and div7a-loan-review 0.3.2, and record both unpublished versions
in each release note.

The three workbooks are rebuilt with the desktop Excel pass and differ
only in their two version cells. The MCP's div7a test and quick-proof
transcript follow the workspace engine to 0.3.2.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CCB8D2-AD7F-4507-A3D7-AE94E5591817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8C3998-20BC-4251-8797-F24D6E458100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.2.1. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 0.2.2. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1567,7 +1567,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.2.1</t>
+    <t>0.2.2</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Build the ato-benchmark workbook with the Rust builder and remove the Python one
The shipped workbook is rebuilt through desktop Excel by
`cargo run --example build_workbook` (overall REVIEW, as before). Against the
previous workbook its model differs only in the status fills, now shown in
Excel, each sheet's A4 page setup and the engine version, 1.0.0. Every cached
value equals the Python-built, Excel-recalculated reference.

tools/build_workbook.py is deleted. The root test drops its check of the
builder's copied wording, since the builder now imports it, and pins engine
1.0.0. CHANGELOG, CONTRIBUTING and workbooks/README describe the Rust build.
</commit_message>
<xml_diff>
--- a/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
+++ b/packages/ato-benchmark-compare/workbooks/ato-benchmark-compare.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8C3998-20BC-4251-8797-F24D6E458100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2625D32-9F68-433D-92CB-335B94D29FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>ato-benchmark-compare workbook, engine 0.2.2. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>ato-benchmark-compare workbook, engine 1.0.0. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>Account</t>
@@ -1567,7 +1567,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.2.2</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -1677,27 +1677,37 @@
       <sz val="14"/>
       <color rgb="FF5C2D91"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1F4E9E"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1710,16 +1720,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF3F1F6"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF5C2D91"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2E0DF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1767,43 +1780,43 @@
   <dxfs count="6">
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
+        <patternFill>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF3CD"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
+        <patternFill>
+          <bgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
+        <patternFill>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF3CD"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
+        <patternFill>
+          <bgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1821,7 +1834,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblPnl" displayName="tblPnl" ref="A1:F28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblPnl" displayName="tblPnl" ref="A1:F28" totalsRowShown="0">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Account"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Amount"/>
@@ -1843,7 +1856,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblMapping" displayName="tblMapping" ref="A1:E28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblMapping" displayName="tblMapping" ref="A1:E28" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Account"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Bucket"/>
@@ -1858,7 +1871,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblBands" displayName="tblBands" ref="A1:V593">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblBands" displayName="tblBands" ref="A1:V593" totalsRowShown="0">
   <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Year"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Industry"/>
@@ -1888,9 +1901,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1928,7 +1941,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1962,6 +1975,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1996,9 +2010,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2242,6 +2257,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -2925,6 +2941,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -3456,6 +3473,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -33621,6 +33639,7 @@
   </sheetData>
   <sheetProtection sheet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -34002,6 +34021,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
@@ -34247,6 +34267,7 @@
   </sheetData>
   <sheetProtection sheet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -34523,6 +34544,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -34697,5 +34719,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
</xml_diff>